<commit_message>
Brand integration and header logo fixes
</commit_message>
<xml_diff>
--- a/inventory/output/review/review_flags.xlsx
+++ b/inventory/output/review/review_flags.xlsx
@@ -103,7 +103,7 @@
     <t>Review Reason</t>
   </si>
   <si>
-    <t>MRH-0015</t>
+    <t>MRH-0028</t>
   </si>
   <si>
     <t/>
@@ -130,171 +130,171 @@
     <t>2026-05-21T13:49:39.561Z</t>
   </si>
   <si>
+    <t>2026-05-22T21:08:20.458Z</t>
+  </si>
+  <si>
+    <t>dore\WhatsApp Image 2026-05-21 at 10.03.44 AM.jpeg</t>
+  </si>
+  <si>
+    <t>raw/dore</t>
+  </si>
+  <si>
+    <t>2026-05-22T21:08:04.592Z</t>
+  </si>
+  <si>
+    <t>RUN-20260523-023801</t>
+  </si>
+  <si>
+    <t>Missing core: Sector, Property_Type, Rent</t>
+  </si>
+  <si>
+    <t>Needs Review</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 1 BHK | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 1] 1197 [secs2| 402 | zsk [immediately | ar [TY | | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 2| 1197 [secs2| 302 | 25k | 01-06-2026 | 3F | oY | | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: irn ed | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: furnished 0 | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 4] 1534/C | Sec-52| 402 | 26 | Immediately | ar |, to¥ | NOV | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 1RK | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 1|vi2/42|sec24| 203 | 13k | ammediately | sr | "IY | with ie | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 2|vi2/a2 [sec 24] G3 | 16k | immediately] G3 | oY | | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 3|v12/a2[sec24| 301 | 16K | Immediately | TF | “iY | with ie | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: + “soo [ssa] | soc] owas | or || WE | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: “Fully | With | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 7] 1410 [secs2| 305 | 16K | 01-06-2025 | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 8|1533/€ [secs2| 403 | 17k | 10-06-2026 | ar | elY (| NED | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 9 1534/8 [secs2| G2 | 16K | 01-06-2025 | GF | iY | IT) | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: darn ned BaICon | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 13| 560 |secsz |aqunits)| 13k | Tmmediately | |, u¥ | Nh | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: 14] 54123 | Sec-24 [Top floor] 11K | Immediately | 5 | iV | NT | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>Low OCR confidence (58%). Manual review required. Raw line: urnisnca PAICONN | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
+  </si>
+  <si>
+    <t>MRH-0002</t>
+  </si>
+  <si>
+    <t>2bhk</t>
+  </si>
+  <si>
+    <t>Sector 15</t>
+  </si>
+  <si>
+    <t>fnf</t>
+  </si>
+  <si>
+    <t>Raw OCR line: 1 | Rent Ok Sec 15 810 103 Immidiately 2BHK 55K | Score 60/100 (master threshold: 85)</t>
+  </si>
+  <si>
+    <t>fnf\WhatsApp Image 2026-05-20 at 11.48.44 AM.jpeg</t>
+  </si>
+  <si>
+    <t>raw/fnf</t>
+  </si>
+  <si>
+    <t>2026-05-22T21:08:07.240Z</t>
+  </si>
+  <si>
+    <t>Score 60/100 (master threshold: 85)</t>
+  </si>
+  <si>
+    <t>MRH-0003</t>
+  </si>
+  <si>
+    <t>1bhk</t>
+  </si>
+  <si>
+    <t>Sector 38</t>
+  </si>
+  <si>
+    <t>Raw OCR line: 2 | Rent Ok Sec 38 874 301 Immidiately 1BHK | 35K | Score 60/100 (master threshold: 85)</t>
+  </si>
+  <si>
+    <t>MRH-0029</t>
+  </si>
+  <si>
+    <t>1rk</t>
+  </si>
+  <si>
+    <t>Sector 39</t>
+  </si>
+  <si>
+    <t>Raw OCR line: 3 Rent Ok Sec 39 149 303 Immidiately 1RK | 14K | Score 60/100 (master threshold: 85)</t>
+  </si>
+  <si>
+    <t>Raw OCR line: 4 | Rent Ok Sec 39 149 103 Immidiately 1RK | 14K | Score 60/100 (master threshold: 85) | Exact duplicate of a higher-priority record (source: fnf).</t>
+  </si>
+  <si>
+    <t>Raw OCR line: 5 Rent Ok Sec 39 149 406 Immidiately 1RK | 14K | Score 60/100 (master threshold: 85) | Exact duplicate of a higher-priority record (source: fnf).</t>
+  </si>
+  <si>
+    <t>MRH-0030</t>
+  </si>
+  <si>
+    <t>Raw OCR line: 6 Rent Ok Sec 39 755 501 Immidiately 1BHK 35K | Score 60/100 (master threshold: 85)</t>
+  </si>
+  <si>
+    <t>Raw OCR line: 7 Rent Ok Sec 39 755 504 Immidiately 1BHK 35K | Score 60/100 (master threshold: 85) | Exact duplicate of a higher-priority record (source: fnf).</t>
+  </si>
+  <si>
+    <t>MRH-0006</t>
+  </si>
+  <si>
+    <t>Sector 40</t>
+  </si>
+  <si>
+    <t>Raw OCR line: 8 Rent Ok Sec 40 13 103 Immidiately 2BHK 40K | Score 60/100 (master threshold: 85)</t>
+  </si>
+  <si>
+    <t>MRH-0018</t>
+  </si>
+  <si>
+    <t>Sector 43</t>
+  </si>
+  <si>
+    <t>Raw OCR line: 9 Rent Ok Sec 43 EZ 102 Immidiately 2BHK 45K | Score 60/100 (master threshold: 85)</t>
+  </si>
+  <si>
     <t>2026-05-21T14:16:09.283Z</t>
   </si>
   <si>
-    <t>dore\WhatsApp Image 2026-05-21 at 10.03.44 AM.jpeg</t>
-  </si>
-  <si>
-    <t>raw/dore</t>
-  </si>
-  <si>
-    <t>2026-05-21T14:15:50.268Z</t>
-  </si>
-  <si>
-    <t>RUN-20260521-194547</t>
-  </si>
-  <si>
-    <t>Missing core: Sector, Property_Type, Rent</t>
-  </si>
-  <si>
-    <t>Needs Review</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 1 BHK | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 1] 1197 [secs2| 402 | zsk [immediately | ar [TY | | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 2| 1197 [secs2| 302 | 25k | 01-06-2026 | 3F | oY | | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: irn ed | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: furnished 0 | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 4] 1534/C | Sec-52| 402 | 26 | Immediately | ar |, to¥ | NOV | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 1RK | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 1|vi2/42|sec24| 203 | 13k | ammediately | sr | "IY | with ie | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 2|vi2/a2 [sec 24] G3 | 16k | immediately] G3 | oY | | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 3|v12/a2[sec24| 301 | 16K | Immediately | TF | “iY | with ie | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: + “soo [ssa] | soc] owas | or || WE | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: “Fully | With | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 7] 1410 [secs2| 305 | 16K | 01-06-2025 | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 8|1533/€ [secs2| 403 | 17k | 10-06-2026 | ar | elY (| NED | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 9 1534/8 [secs2| G2 | 16K | 01-06-2025 | GF | iY | IT) | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: darn ned BaICon | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 13| 560 |secsz |aqunits)| 13k | Tmmediately | |, u¥ | Nh | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: 14] 54123 | Sec-24 [Top floor] 11K | Immediately | 5 | iV | NT | | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>Low OCR confidence (58%). Manual review required. Raw line: urnisnca PAICONN | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
-  </si>
-  <si>
-    <t>MRH-0002</t>
-  </si>
-  <si>
-    <t>2bhk</t>
-  </si>
-  <si>
-    <t>Sector 15</t>
-  </si>
-  <si>
-    <t>fnf</t>
-  </si>
-  <si>
-    <t>Raw OCR line: 1 | Rent Ok Sec 15 810 103 Immidiately 2BHK 55K | Score 60/100 (master threshold: 85)</t>
-  </si>
-  <si>
-    <t>fnf\WhatsApp Image 2026-05-20 at 11.48.44 AM.jpeg</t>
-  </si>
-  <si>
-    <t>raw/fnf</t>
-  </si>
-  <si>
-    <t>2026-05-21T14:15:53.881Z</t>
-  </si>
-  <si>
-    <t>Score 60/100 (master threshold: 85)</t>
-  </si>
-  <si>
-    <t>MRH-0003</t>
-  </si>
-  <si>
-    <t>1bhk</t>
-  </si>
-  <si>
-    <t>Sector 38</t>
-  </si>
-  <si>
-    <t>Raw OCR line: 2 | Rent Ok Sec 38 874 301 Immidiately 1BHK | 35K | Score 60/100 (master threshold: 85)</t>
-  </si>
-  <si>
-    <t>MRH-0016</t>
-  </si>
-  <si>
-    <t>1rk</t>
-  </si>
-  <si>
-    <t>Sector 39</t>
-  </si>
-  <si>
-    <t>Raw OCR line: 3 Rent Ok Sec 39 149 303 Immidiately 1RK | 14K | Score 60/100 (master threshold: 85)</t>
-  </si>
-  <si>
-    <t>Raw OCR line: 4 | Rent Ok Sec 39 149 103 Immidiately 1RK | 14K | Score 60/100 (master threshold: 85) | Exact duplicate of a higher-priority record (source: fnf).</t>
-  </si>
-  <si>
-    <t>Raw OCR line: 5 Rent Ok Sec 39 149 406 Immidiately 1RK | 14K | Score 60/100 (master threshold: 85) | Exact duplicate of a higher-priority record (source: fnf).</t>
-  </si>
-  <si>
-    <t>MRH-0017</t>
-  </si>
-  <si>
-    <t>Raw OCR line: 6 Rent Ok Sec 39 755 501 Immidiately 1BHK 35K | Score 60/100 (master threshold: 85)</t>
-  </si>
-  <si>
-    <t>Raw OCR line: 7 Rent Ok Sec 39 755 504 Immidiately 1BHK 35K | Score 60/100 (master threshold: 85) | Exact duplicate of a higher-priority record (source: fnf).</t>
-  </si>
-  <si>
-    <t>MRH-0006</t>
-  </si>
-  <si>
-    <t>Sector 40</t>
-  </si>
-  <si>
-    <t>Raw OCR line: 8 Rent Ok Sec 40 13 103 Immidiately 2BHK 40K | Score 60/100 (master threshold: 85)</t>
-  </si>
-  <si>
-    <t>MRH-0018</t>
-  </si>
-  <si>
-    <t>Sector 43</t>
-  </si>
-  <si>
-    <t>Raw OCR line: 9 Rent Ok Sec 43 EZ 102 Immidiately 2BHK 45K | Score 60/100 (master threshold: 85)</t>
-  </si>
-  <si>
-    <t>NEW</t>
-  </si>
-  <si>
     <t>MRH-0019</t>
   </si>
   <si>
@@ -364,13 +364,13 @@
     <t>Raw OCR line: 17 | Rent Ok Sec 51 1222 G002 Immidiately 1BHK 38K | Score 60/100 (master threshold: 85)</t>
   </si>
   <si>
-    <t>MRH-0024</t>
+    <t>MRH-0031</t>
   </si>
   <si>
     <t>Raw OCR line: 18 Rent Ok Sec 51 1222 101 Immidiately 1BHK 38K | Score 60/100 (master threshold: 85)</t>
   </si>
   <si>
-    <t>MRH-0025</t>
+    <t>MRH-0032</t>
   </si>
   <si>
     <t>Raw OCR line: 19 Rent Ok 103 Immidiately 1BHK 38K | Missing core: Sector</t>
@@ -397,7 +397,7 @@
     <t>Raw OCR line: 25 Rent Ok 502 Immidiately 1BHK 35K | Missing core: Sector | Exact duplicate of a higher-priority record (source: fnf).</t>
   </si>
   <si>
-    <t>MRH-0026</t>
+    <t>MRH-0033</t>
   </si>
   <si>
     <t>preoccupied</t>
@@ -418,7 +418,7 @@
     <t>raw/s2l</t>
   </si>
   <si>
-    <t>2026-05-21T14:15:59.953Z</t>
+    <t>2026-05-22T21:08:11.457Z</t>
   </si>
   <si>
     <t>Raw OCR line: | 3 | sees2 | 203 | 1787 | immediately | Preoccupied | 21K | Missing core: Sector | Exact duplicate of a higher-priority record (source: s2l).</t>
@@ -463,7 +463,7 @@
     <t>s2l\WhatsApp Image 2026-05-21 at 12.06.13 PM.jpeg</t>
   </si>
   <si>
-    <t>2026-05-21T14:16:09.255Z</t>
+    <t>2026-05-22T21:08:20.444Z</t>
   </si>
   <si>
     <t>Low OCR confidence (59%). Manual review required. Raw line: Sr.No Vacating Type | Missing core: Sector, Property_Type, Rent | Exact duplicate of a higher-priority record (source: dore).</t>
@@ -3885,10 +3885,10 @@
         <v>92</v>
       </c>
       <c r="V31" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W31" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W31" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X31" s="4" t="s">
         <v>39</v>
@@ -3977,10 +3977,10 @@
         <v>96</v>
       </c>
       <c r="V32" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W32" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W32" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X32" s="4" t="s">
         <v>39</v>
@@ -4345,10 +4345,10 @@
         <v>105</v>
       </c>
       <c r="V36" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W36" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W36" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X36" s="4" t="s">
         <v>39</v>
@@ -4437,10 +4437,10 @@
         <v>109</v>
       </c>
       <c r="V37" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W37" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W37" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X37" s="4" t="s">
         <v>39</v>
@@ -4529,10 +4529,10 @@
         <v>112</v>
       </c>
       <c r="V38" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W38" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W38" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X38" s="4" t="s">
         <v>39</v>
@@ -4621,10 +4621,10 @@
         <v>116</v>
       </c>
       <c r="V39" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W39" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W39" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X39" s="4" t="s">
         <v>39</v>
@@ -4713,10 +4713,10 @@
         <v>118</v>
       </c>
       <c r="V40" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W40" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W40" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X40" s="4" t="s">
         <v>39</v>
@@ -4897,10 +4897,10 @@
         <v>122</v>
       </c>
       <c r="V42" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W42" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W42" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X42" s="4" t="s">
         <v>39</v>
@@ -5449,10 +5449,10 @@
         <v>132</v>
       </c>
       <c r="V48" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W48" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W48" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X48" s="4" t="s">
         <v>39</v>
@@ -5541,10 +5541,10 @@
         <v>136</v>
       </c>
       <c r="V49" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W49" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W49" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X49" s="4" t="s">
         <v>39</v>
@@ -6369,10 +6369,10 @@
         <v>147</v>
       </c>
       <c r="V58" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W58" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="W58" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="X58" s="4" t="s">
         <v>39</v>

</xml_diff>